<commit_message>
updated project code 1
</commit_message>
<xml_diff>
--- a/TestData1/AutoExtendFile.xlsx
+++ b/TestData1/AutoExtendFile.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="5">
   <si>
     <t>eway_bill_number</t>
   </si>
@@ -63,6 +63,9 @@
 Command: [695f9328ff86f17e4c807eb733309a40, get {url=https://ewaybillgst.gov.in/MainMenu.aspx}]
 Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 152.0.7977.65, chrome: {chromedriverVersion: 152.0.7977.64 (506c834eccea..., userDataDir: C:\Users\kasif\AppData\Loca...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:56332}, goog:processID: 6708, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:56332/devtoo..., se:cdpVersion: 152.0.7977.65, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
 Session ID: 695f9328ff86f17e4c807eb733309a40</t>
+  </si>
+  <si>
+    <t>Extended (Valid Until: 06/09/2026)</t>
   </si>
 </sst>
 </file>
@@ -552,7 +555,7 @@
         <v>592040564957</v>
       </c>
       <c r="B13" t="s" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
@@ -560,7 +563,7 @@
         <v>562041080862</v>
       </c>
       <c r="B14" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
@@ -568,7 +571,7 @@
         <v>542039971499</v>
       </c>
       <c r="B15" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
@@ -576,7 +579,7 @@
         <v>411750413493</v>
       </c>
       <c r="B16" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
@@ -584,7 +587,7 @@
         <v>491750835956</v>
       </c>
       <c r="B17" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
@@ -592,7 +595,7 @@
         <v>411746014750</v>
       </c>
       <c r="B18" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
@@ -600,7 +603,7 @@
         <v>451748588239</v>
       </c>
       <c r="B19" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
@@ -608,7 +611,7 @@
         <v>491749397483</v>
       </c>
       <c r="B20" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
@@ -616,7 +619,7 @@
         <v>421751477938</v>
       </c>
       <c r="B21" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
@@ -624,7 +627,7 @@
         <v>461751380216</v>
       </c>
       <c r="B22" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
@@ -632,7 +635,7 @@
         <v>411751477344</v>
       </c>
       <c r="B23" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
@@ -640,7 +643,7 @@
         <v>481751225447</v>
       </c>
       <c r="B24" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
@@ -648,7 +651,7 @@
         <v>401751226855</v>
       </c>
       <c r="B25" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
@@ -656,7 +659,7 @@
         <v>401747349054</v>
       </c>
       <c r="B26" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
@@ -664,7 +667,7 @@
         <v>481751226820</v>
       </c>
       <c r="B27" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
@@ -672,7 +675,7 @@
         <v>172479422761</v>
       </c>
       <c r="B28" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
@@ -680,7 +683,7 @@
         <v>481745690482</v>
       </c>
       <c r="B29" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
@@ -688,7 +691,7 @@
         <v>471750228262</v>
       </c>
       <c r="B30" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
@@ -696,7 +699,7 @@
         <v>471749809487</v>
       </c>
       <c r="B31" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
@@ -704,7 +707,7 @@
         <v>282247192056</v>
       </c>
       <c r="B32" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
@@ -712,7 +715,7 @@
         <v>252246797189</v>
       </c>
       <c r="B33" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
@@ -720,7 +723,7 @@
         <v>212246080876</v>
       </c>
       <c r="B34" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
@@ -728,7 +731,7 @@
         <v>801700106728</v>
       </c>
       <c r="B35" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
@@ -736,7 +739,7 @@
         <v>888009472101</v>
       </c>
       <c r="B36" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
@@ -744,7 +747,7 @@
         <v>801700103422</v>
       </c>
       <c r="B37" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
@@ -752,7 +755,7 @@
         <v>888009494415</v>
       </c>
       <c r="B38" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
@@ -760,7 +763,7 @@
         <v>818009494401</v>
       </c>
       <c r="B39" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
@@ -768,7 +771,7 @@
         <v>821700990565</v>
       </c>
       <c r="B40" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
@@ -776,7 +779,7 @@
         <v>861700989619</v>
       </c>
       <c r="B41" t="s" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
@@ -784,7 +787,7 @@
         <v>572034573794</v>
       </c>
       <c r="B42" t="s" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">

</xml_diff>